<commit_message>
Rename to MNOffice, part of Mundus Novus
New icons and palette, office.mundusnovus.org, the MNOffice desktop app,
and the writing font renamed Novus Serif (rebuilt from Liberation Serif,
OFL) with the blank templates updated to use it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portal/templates/blank.xlsx
+++ b/portal/templates/blank.xlsx
@@ -24,7 +24,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Christian Sans"/>
+      <name val="Novus Serif"/>
       <family val="2"/>
       <charset val="204"/>
       <scheme val="minor"/>
@@ -119,8 +119,8 @@
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Christian Sans"/>
-        <a:font script="Hebr" typeface="Christian Sans"/>
+        <a:font script="Arab" typeface="Novus Serif"/>
+        <a:font script="Hebr" typeface="Novus Serif"/>
         <a:font script="Thai" typeface="Tahoma"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
@@ -142,20 +142,20 @@
         <a:font script="Laoo" typeface="DokChampa"/>
         <a:font script="Sinh" typeface="Iskoola Pota"/>
         <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Christian Sans"/>
+        <a:font script="Viet" typeface="Novus Serif"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Christian Sans" panose="020F0502020204030204"/>
+        <a:latin typeface="Novus Serif" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Christian Sans"/>
-        <a:font script="Hebr" typeface="Christian Sans"/>
+        <a:font script="Arab" typeface="Novus Serif"/>
+        <a:font script="Hebr" typeface="Novus Serif"/>
         <a:font script="Thai" typeface="Tahoma"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
@@ -177,7 +177,7 @@
         <a:font script="Laoo" typeface="DokChampa"/>
         <a:font script="Sinh" typeface="Iskoola Pota"/>
         <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Christian Sans"/>
+        <a:font script="Viet" typeface="Novus Serif"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>

</xml_diff>

<commit_message>
Rename to Asteria Office, part of Asteria Technology
New name, asteria.technology addresses, the teal palette and the new icons,
fonts renamed Asteria Pixel and Asteria Serif, and the Asteria License.
Settings and files saved under the earlier names still load.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portal/templates/blank.xlsx
+++ b/portal/templates/blank.xlsx
@@ -24,7 +24,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Novus Serif"/>
+      <name val="Asteria Serif"/>
       <family val="2"/>
       <charset val="204"/>
       <scheme val="minor"/>
@@ -119,8 +119,8 @@
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Novus Serif"/>
-        <a:font script="Hebr" typeface="Novus Serif"/>
+        <a:font script="Arab" typeface="Asteria Serif"/>
+        <a:font script="Hebr" typeface="Asteria Serif"/>
         <a:font script="Thai" typeface="Tahoma"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
@@ -142,20 +142,20 @@
         <a:font script="Laoo" typeface="DokChampa"/>
         <a:font script="Sinh" typeface="Iskoola Pota"/>
         <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Novus Serif"/>
+        <a:font script="Viet" typeface="Asteria Serif"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Novus Serif" panose="020F0502020204030204"/>
+        <a:latin typeface="Asteria Serif" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Novus Serif"/>
-        <a:font script="Hebr" typeface="Novus Serif"/>
+        <a:font script="Arab" typeface="Asteria Serif"/>
+        <a:font script="Hebr" typeface="Asteria Serif"/>
         <a:font script="Thai" typeface="Tahoma"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
@@ -177,7 +177,7 @@
         <a:font script="Laoo" typeface="DokChampa"/>
         <a:font script="Sinh" typeface="Iskoola Pota"/>
         <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Novus Serif"/>
+        <a:font script="Viet" typeface="Asteria Serif"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>

</xml_diff>